<commit_message>
feat: audited cleaning, implemented research log
Major overhaul of `01_data-cleaning.qmd` to establish a self-validating data prep workflow.

Key changes:
- **Renaming Logic:** Separated variable renaming (structural) from data type conversion (encoding) to allow for 1:1 integrity checks.
- **Auditing:** Refined semi-automated audit functions to verify longitudinal data completeness and naming consistency.
- **Integrity Checks:** Implemented reverse-traceability checks to confirm clean variables map correctly to raw columns.
- **Documentation:** Added `docs/research_log.md` for issue tracking and in-script callouts for immediate context on data anomalies.
- **Artifacts:** Configured script to save `gic_renamed.rds` for validation in the next pipeline stage.

Refactored:
- Replaced manual `identical()` checks with single tibble table.
- Standardized all variable names to snake_case (`stem_#` format).
</commit_message>
<xml_diff>
--- a/docs/glossary.xlsx
+++ b/docs/glossary.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olucdenver.sharepoint.com/sites/HendricksLabDailyWorkSpace/Shared Documents/Research Projects/Tinashe Collaborations/gi-cancer_project/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{074114E1-AEC4-440E-9A9F-2F76837AA4D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09D1CC24-F320-416B-A196-E14CBD1E85CF}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="8_{074114E1-AEC4-440E-9A9F-2F76837AA4D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68FBD7D4-F2BC-43E1-A2AC-05F333589984}"/>
   <bookViews>
-    <workbookView xWindow="47964" yWindow="2028" windowWidth="34560" windowHeight="18600" xr2:uid="{2AF94D29-0516-4E66-985C-E773281D9243}"/>
+    <workbookView xWindow="5640" yWindow="2448" windowWidth="34560" windowHeight="18600" xr2:uid="{2AF94D29-0516-4E66-985C-E773281D9243}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$71</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="236">
   <si>
     <t>Variable</t>
   </si>
@@ -104,12 +104,6 @@
     <t>hx_cancer</t>
   </si>
   <si>
-    <t>weight</t>
-  </si>
-  <si>
-    <t>height</t>
-  </si>
-  <si>
     <t>tx_concurrent_rtx</t>
   </si>
   <si>
@@ -128,9 +122,6 @@
     <t>cycles_given</t>
   </si>
   <si>
-    <t>completion_rate_pct</t>
-  </si>
-  <si>
     <t>death_date</t>
   </si>
   <si>
@@ -257,27 +248,6 @@
     <t>Family history of cancer</t>
   </si>
   <si>
-    <t>bmi_#</t>
-  </si>
-  <si>
-    <t>cd4_count_#</t>
-  </si>
-  <si>
-    <t>urea_#</t>
-  </si>
-  <si>
-    <t>creat_#</t>
-  </si>
-  <si>
-    <t>cr_clear_#</t>
-  </si>
-  <si>
-    <t>cea_#</t>
-  </si>
-  <si>
-    <t>ca199_#</t>
-  </si>
-  <si>
     <t>orig_order</t>
   </si>
   <si>
@@ -302,9 +272,6 @@
     <t>Date of death (if death occurred)</t>
   </si>
   <si>
-    <t>**Biomarkers**</t>
-  </si>
-  <si>
     <t>Numeric</t>
   </si>
   <si>
@@ -638,9 +605,6 @@
     <t>CD4+ T-cell count</t>
   </si>
   <si>
-    <t>albi_score_#</t>
-  </si>
-  <si>
     <t>Cycle delayed due to toxicity</t>
   </si>
   <si>
@@ -735,6 +699,54 @@
   </si>
   <si>
     <t>**Ref:** 18.5 - 24.9 &lt;sup&gt;[1]&lt;/sup&gt;</t>
+  </si>
+  <si>
+    <t>completion_rate</t>
+  </si>
+  <si>
+    <t>bmi_0</t>
+  </si>
+  <si>
+    <t>cd4_count_0</t>
+  </si>
+  <si>
+    <t>urea_0</t>
+  </si>
+  <si>
+    <t>creat_0</t>
+  </si>
+  <si>
+    <t>cr_clear_0</t>
+  </si>
+  <si>
+    <t>albi_score_0</t>
+  </si>
+  <si>
+    <t>cea_0</t>
+  </si>
+  <si>
+    <t>ca199_0</t>
+  </si>
+  <si>
+    <t>**Longitudinal - Hematology**</t>
+  </si>
+  <si>
+    <t>**Longitudinal - Chemistry**</t>
+  </si>
+  <si>
+    <t>**Longitudinal - Liver Function**</t>
+  </si>
+  <si>
+    <t>**Longitudinal - Management**</t>
+  </si>
+  <si>
+    <t>**Baseline-Only Measurements**</t>
+  </si>
+  <si>
+    <t>weight_0</t>
+  </si>
+  <si>
+    <t>height_0</t>
   </si>
 </sst>
 </file>
@@ -1141,7 +1153,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60F3F596-38F5-43D0-B51C-7C799C94B00A}">
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.5546875" bestFit="1" customWidth="1"/>
@@ -1156,27 +1168,27 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="C1" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="D1" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
       <c r="E1" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="F1" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="G1" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="G2" s="1">
         <v>1</v>
@@ -1187,16 +1199,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D3" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="E3" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -1210,16 +1222,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D4" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="E4" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="F4">
         <v>2</v>
@@ -1230,7 +1242,7 @@
     </row>
     <row r="5" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="G5" s="1">
         <v>4</v>
@@ -1241,16 +1253,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C6" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D6" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="E6" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F6">
         <v>4</v>
@@ -1264,16 +1276,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C7" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D7" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="E7" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="F7">
         <v>5</v>
@@ -1284,7 +1296,7 @@
     </row>
     <row r="8" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="G8" s="1">
         <v>7</v>
@@ -1295,16 +1307,16 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="C9" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D9" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="E9" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="F9">
         <v>3</v>
@@ -1318,16 +1330,16 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C10" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D10" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="E10" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="F10">
         <v>6</v>
@@ -1341,21 +1353,21 @@
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D11" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="E11" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="F11">
         <v>7</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="1">
         <v>10</v>
       </c>
     </row>
@@ -1364,16 +1376,16 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="C12" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D12" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="E12" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="F12">
         <v>8</v>
@@ -1384,19 +1396,19 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="C13" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D13" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E13" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="F13">
         <v>46</v>
@@ -1407,42 +1419,42 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="C14" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D14" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="E14" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="F14">
         <v>47</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="1">
         <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="C15" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D15" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="E15" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="F15">
         <v>48</v>
@@ -1453,19 +1465,19 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="C16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D16" t="s">
         <v>174</v>
       </c>
-      <c r="D16" t="s">
-        <v>185</v>
-      </c>
       <c r="E16" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="F16">
         <v>49</v>
@@ -1476,42 +1488,42 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="C17" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D17" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="E17" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="F17">
         <v>50</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="1">
         <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="C18" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D18" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="E18" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="F18">
         <v>51</v>
@@ -1522,19 +1534,19 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>220</v>
       </c>
       <c r="B19" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="C19" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D19" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="E19" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="F19">
         <v>52</v>
@@ -1545,7 +1557,7 @@
     </row>
     <row r="20" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="G20" s="1">
         <v>19</v>
@@ -1556,16 +1568,16 @@
         <v>9</v>
       </c>
       <c r="B21" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C21" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D21" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E21" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="F21">
         <v>9</v>
@@ -1579,16 +1591,16 @@
         <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C22" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D22" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E22" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="F22">
         <v>10</v>
@@ -1602,21 +1614,21 @@
         <v>11</v>
       </c>
       <c r="B23" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C23" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D23" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E23" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="F23">
         <v>11</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="1">
         <v>22</v>
       </c>
     </row>
@@ -1625,16 +1637,16 @@
         <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C24" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D24" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E24" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="F24">
         <v>12</v>
@@ -1648,16 +1660,16 @@
         <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C25" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D25" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E25" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="F25">
         <v>13</v>
@@ -1671,21 +1683,21 @@
         <v>14</v>
       </c>
       <c r="B26" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C26" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D26" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E26" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="F26">
         <v>14</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="1">
         <v>25</v>
       </c>
     </row>
@@ -1694,16 +1706,16 @@
         <v>15</v>
       </c>
       <c r="B27" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C27" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D27" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E27" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="F27">
         <v>15</v>
@@ -1717,16 +1729,16 @@
         <v>16</v>
       </c>
       <c r="B28" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C28" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D28" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E28" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="F28">
         <v>16</v>
@@ -1740,21 +1752,21 @@
         <v>17</v>
       </c>
       <c r="B29" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C29" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D29" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E29" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="F29">
         <v>17</v>
       </c>
-      <c r="G29">
+      <c r="G29" s="1">
         <v>28</v>
       </c>
     </row>
@@ -1763,16 +1775,16 @@
         <v>18</v>
       </c>
       <c r="B30" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C30" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D30" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E30" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="F30">
         <v>18</v>
@@ -1786,16 +1798,16 @@
         <v>19</v>
       </c>
       <c r="B31" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C31" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D31" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E31" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="F31">
         <v>19</v>
@@ -1809,65 +1821,50 @@
         <v>20</v>
       </c>
       <c r="B32" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C32" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D32" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E32" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="F32">
         <v>20</v>
       </c>
-      <c r="G32">
+      <c r="G32" s="1">
         <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B33" t="s">
-        <v>169</v>
+        <v>76</v>
       </c>
       <c r="C33" t="s">
-        <v>88</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>220</v>
+        <v>164</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>179</v>
       </c>
       <c r="E33" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="F33">
-        <v>21</v>
+        <v>78</v>
       </c>
       <c r="G33">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>22</v>
-      </c>
-      <c r="B34" t="s">
-        <v>160</v>
-      </c>
-      <c r="C34" t="s">
-        <v>88</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="E34" t="s">
-        <v>112</v>
-      </c>
-      <c r="F34">
-        <v>22</v>
+    <row r="34" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>233</v>
       </c>
       <c r="G34">
         <v>33</v>
@@ -1875,96 +1872,111 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>30</v>
+        <v>234</v>
       </c>
       <c r="B35" t="s">
-        <v>86</v>
+        <v>158</v>
       </c>
       <c r="C35" t="s">
-        <v>175</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>190</v>
+        <v>77</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>208</v>
       </c>
       <c r="E35" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="F35">
-        <v>78</v>
-      </c>
-      <c r="G35">
+        <v>21</v>
+      </c>
+      <c r="G35" s="1">
         <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>72</v>
+        <v>235</v>
       </c>
       <c r="B36" t="s">
-        <v>80</v>
+        <v>149</v>
       </c>
       <c r="C36" t="s">
-        <v>88</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>231</v>
+        <v>77</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>208</v>
       </c>
       <c r="E36" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="F36">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G36">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="G37" s="1">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>221</v>
+      </c>
+      <c r="B37" t="s">
+        <v>70</v>
+      </c>
+      <c r="C37" t="s">
+        <v>77</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="E37" t="s">
+        <v>102</v>
+      </c>
+      <c r="F37">
+        <v>23</v>
+      </c>
+      <c r="G37">
         <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>73</v>
+        <v>222</v>
       </c>
       <c r="B38" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="C38" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="E38" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="F38">
         <v>27</v>
       </c>
-      <c r="G38">
+      <c r="G38" s="1">
         <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>74</v>
+        <v>223</v>
       </c>
       <c r="B39" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="C39" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="E39" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="F39">
         <v>33</v>
@@ -1975,19 +1987,19 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>75</v>
+        <v>224</v>
       </c>
       <c r="B40" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="C40" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="E40" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="F40">
         <v>34</v>
@@ -1998,42 +2010,42 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>76</v>
+        <v>225</v>
       </c>
       <c r="B41" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="C41" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="E41" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="F41">
         <v>35</v>
       </c>
-      <c r="G41">
+      <c r="G41" s="1">
         <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>199</v>
+        <v>226</v>
       </c>
       <c r="B42" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="C42" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="E42" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F42">
         <v>43</v>
@@ -2044,19 +2056,19 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>77</v>
+        <v>227</v>
       </c>
       <c r="B43" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="C43" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="E43" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="F43">
         <v>44</v>
@@ -2067,45 +2079,30 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>78</v>
+        <v>228</v>
       </c>
       <c r="B44" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="C44" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="E44" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="F44">
         <v>45</v>
       </c>
-      <c r="G44">
+      <c r="G44" s="1">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>39</v>
-      </c>
-      <c r="B45" t="s">
-        <v>210</v>
-      </c>
-      <c r="C45" t="s">
-        <v>88</v>
-      </c>
-      <c r="D45" t="s">
-        <v>214</v>
-      </c>
-      <c r="E45" t="s">
-        <v>146</v>
-      </c>
-      <c r="F45">
-        <v>37</v>
+    <row r="45" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>229</v>
       </c>
       <c r="G45">
         <v>44</v>
@@ -2113,22 +2110,22 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="B46" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="C46" t="s">
-        <v>88</v>
-      </c>
-      <c r="D46" t="s">
-        <v>215</v>
+        <v>77</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>200</v>
       </c>
       <c r="E46" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="F46">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="G46">
         <v>45</v>
@@ -2136,45 +2133,45 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="B47" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C47" t="s">
-        <v>88</v>
-      </c>
-      <c r="D47" t="s">
-        <v>216</v>
+        <v>77</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>201</v>
       </c>
       <c r="E47" t="s">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="F47">
-        <v>41</v>
-      </c>
-      <c r="G47">
+        <v>29</v>
+      </c>
+      <c r="G47" s="1">
         <v>46</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B48" t="s">
-        <v>211</v>
+        <v>152</v>
       </c>
       <c r="C48" t="s">
-        <v>88</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>217</v>
+        <v>77</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>201</v>
       </c>
       <c r="E48" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="F48">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G48">
         <v>47</v>
@@ -2182,22 +2179,22 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="B49" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C49" t="s">
-        <v>88</v>
-      </c>
-      <c r="D49" t="s">
-        <v>218</v>
+        <v>77</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>209</v>
       </c>
       <c r="E49" t="s">
-        <v>149</v>
+        <v>128</v>
       </c>
       <c r="F49">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="G49">
         <v>48</v>
@@ -2205,45 +2202,45 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="B50" t="s">
-        <v>158</v>
+        <v>141</v>
       </c>
       <c r="C50" t="s">
-        <v>88</v>
-      </c>
-      <c r="D50" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D50" s="3" t="s">
         <v>213</v>
       </c>
       <c r="E50" t="s">
-        <v>131</v>
+        <v>103</v>
       </c>
       <c r="F50">
-        <v>67</v>
-      </c>
-      <c r="G50">
+        <v>24</v>
+      </c>
+      <c r="G50" s="1">
         <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="B51" t="s">
-        <v>159</v>
+        <v>199</v>
       </c>
       <c r="C51" t="s">
-        <v>88</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>213</v>
+        <v>77</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>205</v>
       </c>
       <c r="E51" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="F51">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="G51">
         <v>50</v>
@@ -2251,68 +2248,53 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B52" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
       <c r="C52" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="E52" t="s">
-        <v>140</v>
+        <v>119</v>
       </c>
       <c r="F52">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="G52">
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>37</v>
-      </c>
-      <c r="B53" t="s">
-        <v>162</v>
-      </c>
-      <c r="C53" t="s">
-        <v>88</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="E53" t="s">
-        <v>130</v>
-      </c>
-      <c r="F53">
-        <v>60</v>
-      </c>
-      <c r="G53">
+    <row r="53" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="G53" s="1">
         <v>52</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="B54" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C54" t="s">
-        <v>88</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>213</v>
+        <v>77</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>211</v>
       </c>
       <c r="E54" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="F54">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G54">
         <v>53</v>
@@ -2320,68 +2302,53 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
+        <v>44</v>
+      </c>
+      <c r="B55" t="s">
+        <v>155</v>
+      </c>
+      <c r="C55" t="s">
+        <v>77</v>
+      </c>
+      <c r="D55" t="s">
+        <v>210</v>
+      </c>
+      <c r="E55" t="s">
+        <v>133</v>
+      </c>
+      <c r="F55">
         <v>32</v>
-      </c>
-      <c r="B55" t="s">
-        <v>164</v>
-      </c>
-      <c r="C55" t="s">
-        <v>88</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="E55" t="s">
-        <v>141</v>
-      </c>
-      <c r="F55">
-        <v>29</v>
       </c>
       <c r="G55">
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>34</v>
-      </c>
-      <c r="B56" t="s">
-        <v>165</v>
-      </c>
-      <c r="C56" t="s">
-        <v>88</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="E56" t="s">
-        <v>139</v>
-      </c>
-      <c r="F56">
-        <v>26</v>
-      </c>
-      <c r="G56">
+    <row r="56" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="G56" s="1">
         <v>55</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="B57" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="C57" t="s">
-        <v>88</v>
-      </c>
-      <c r="D57" t="s">
-        <v>222</v>
+        <v>77</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>201</v>
       </c>
       <c r="E57" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="F57">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G57">
         <v>56</v>
@@ -2389,22 +2356,22 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="B58" t="s">
-        <v>170</v>
+        <v>198</v>
       </c>
       <c r="C58" t="s">
-        <v>88</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>223</v>
+        <v>77</v>
+      </c>
+      <c r="D58" t="s">
+        <v>202</v>
       </c>
       <c r="E58" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="F58">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="G58">
         <v>57</v>
@@ -2412,24 +2379,24 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B59" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="C59" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D59" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="E59" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="F59">
         <v>38</v>
       </c>
-      <c r="G59">
+      <c r="G59" s="1">
         <v>58</v>
       </c>
     </row>
@@ -2438,19 +2405,19 @@
         <v>38</v>
       </c>
       <c r="B60" t="s">
-        <v>168</v>
+        <v>147</v>
       </c>
       <c r="C60" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="E60" t="s">
-        <v>145</v>
+        <v>120</v>
       </c>
       <c r="F60">
-        <v>36</v>
+        <v>67</v>
       </c>
       <c r="G60">
         <v>59</v>
@@ -2458,22 +2425,22 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B61" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="C61" t="s">
-        <v>88</v>
-      </c>
-      <c r="D61" s="3" t="s">
-        <v>225</v>
+        <v>77</v>
+      </c>
+      <c r="D61" t="s">
+        <v>203</v>
       </c>
       <c r="E61" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="F61">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="G61">
         <v>60</v>
@@ -2481,45 +2448,45 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B62" t="s">
-        <v>200</v>
+        <v>144</v>
       </c>
       <c r="C62" t="s">
-        <v>174</v>
+        <v>77</v>
       </c>
       <c r="D62" t="s">
-        <v>186</v>
+        <v>204</v>
       </c>
       <c r="E62" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="F62">
-        <v>72</v>
-      </c>
-      <c r="G62">
+        <v>41</v>
+      </c>
+      <c r="G62" s="1">
         <v>61</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B63" t="s">
-        <v>201</v>
+        <v>145</v>
       </c>
       <c r="C63" t="s">
-        <v>174</v>
+        <v>77</v>
       </c>
       <c r="D63" t="s">
-        <v>186</v>
+        <v>206</v>
       </c>
       <c r="E63" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="F63">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="G63">
         <v>62</v>
@@ -2527,68 +2494,53 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B64" t="s">
-        <v>202</v>
+        <v>148</v>
       </c>
       <c r="C64" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>220</v>
+        <v>201</v>
       </c>
       <c r="E64" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="F64">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="G64">
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>51</v>
-      </c>
-      <c r="B65" t="s">
-        <v>203</v>
-      </c>
-      <c r="C65" t="s">
-        <v>174</v>
-      </c>
-      <c r="D65" t="s">
-        <v>186</v>
-      </c>
-      <c r="E65" t="s">
-        <v>135</v>
-      </c>
-      <c r="F65">
-        <v>75</v>
-      </c>
-      <c r="G65">
+    <row r="65" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="G65" s="1">
         <v>64</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="B66" t="s">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="C66" t="s">
-        <v>88</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>220</v>
+        <v>163</v>
+      </c>
+      <c r="D66" t="s">
+        <v>175</v>
       </c>
       <c r="E66" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="F66">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="G66">
         <v>65</v>
@@ -2596,56 +2548,148 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B67" t="s">
-        <v>205</v>
+        <v>189</v>
       </c>
       <c r="C67" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D67" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="E67" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="F67">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G67">
         <v>66</v>
       </c>
     </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>47</v>
+      </c>
+      <c r="B68" t="s">
+        <v>190</v>
+      </c>
+      <c r="C68" t="s">
+        <v>77</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E68" t="s">
+        <v>123</v>
+      </c>
+      <c r="F68">
+        <v>74</v>
+      </c>
+      <c r="G68" s="1">
+        <v>67</v>
+      </c>
+    </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D69" s="3" t="s">
-        <v>226</v>
+      <c r="A69" t="s">
+        <v>48</v>
+      </c>
+      <c r="B69" t="s">
+        <v>191</v>
+      </c>
+      <c r="C69" t="s">
+        <v>163</v>
+      </c>
+      <c r="D69" t="s">
+        <v>175</v>
+      </c>
+      <c r="E69" t="s">
+        <v>124</v>
+      </c>
+      <c r="F69">
+        <v>75</v>
+      </c>
+      <c r="G69">
+        <v>68</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>49</v>
+      </c>
+      <c r="B70" t="s">
+        <v>192</v>
+      </c>
+      <c r="C70" t="s">
+        <v>77</v>
+      </c>
       <c r="D70" s="2" t="s">
-        <v>227</v>
+        <v>208</v>
+      </c>
+      <c r="E70" t="s">
+        <v>125</v>
+      </c>
+      <c r="F70">
+        <v>76</v>
+      </c>
+      <c r="G70">
+        <v>69</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D71" s="4" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D72" s="5" t="s">
-        <v>229</v>
+      <c r="A71" t="s">
+        <v>50</v>
+      </c>
+      <c r="B71" t="s">
+        <v>193</v>
+      </c>
+      <c r="C71" t="s">
+        <v>163</v>
+      </c>
+      <c r="D71" t="s">
+        <v>175</v>
+      </c>
+      <c r="E71" t="s">
+        <v>126</v>
+      </c>
+      <c r="F71">
+        <v>77</v>
+      </c>
+      <c r="G71" s="1">
+        <v>70</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D73" t="s">
-        <v>230</v>
+      <c r="D73" s="3" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D74" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D75" s="4" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D76" s="5" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D77" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G67" xr:uid="{60F3F596-38F5-43D0-B51C-7C799C94B00A}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A45:G61">
-    <sortCondition ref="A45:A61"/>
+  <autoFilter ref="A1:G71" xr:uid="{60F3F596-38F5-43D0-B51C-7C799C94B00A}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A64:G64">
+    <sortCondition ref="A64"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2887,6 +2931,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="44ad9495-3741-4708-b440-876241155999">
@@ -2895,15 +2948,6 @@
     <TaxCatchAll xmlns="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2926,6 +2970,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{351A9940-6E89-4EED-A102-125C210064C4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05141117-6D65-4604-9391-C80E4C64FB19}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2934,12 +2986,4 @@
     <ds:schemaRef ds:uri="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{351A9940-6E89-4EED-A102-125C210064C4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(data): encode variables and add type audits
Converted all static and longitudinal variables to correct R types including Factors, Dates, and Numerics.

Added a four-part pre/post audit system to verify integrity across static and cyclic variables using numeric tolerance checks and factor mapping verification.

Updated research_log.md with new anomalies found during the encoding process.
</commit_message>
<xml_diff>
--- a/docs/glossary.xlsx
+++ b/docs/glossary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olucdenver.sharepoint.com/sites/HendricksLabDailyWorkSpace/Shared Documents/Research Projects/Tinashe Collaborations/gi-cancer_project/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="8_{074114E1-AEC4-440E-9A9F-2F76837AA4D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68FBD7D4-F2BC-43E1-A2AC-05F333589984}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="8_{074114E1-AEC4-440E-9A9F-2F76837AA4D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5837F166-8F3C-4710-B010-6AD1C8B582A4}"/>
   <bookViews>
-    <workbookView xWindow="5640" yWindow="2448" windowWidth="34560" windowHeight="18600" xr2:uid="{2AF94D29-0516-4E66-985C-E773281D9243}"/>
+    <workbookView xWindow="61152" yWindow="3192" windowWidth="34560" windowHeight="18600" xr2:uid="{2AF94D29-0516-4E66-985C-E773281D9243}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="236">
   <si>
     <t>Variable</t>
   </si>
@@ -635,9 +635,6 @@
     <t>Serum creatinine</t>
   </si>
   <si>
-    <t>Srum Albumin (g/L)</t>
-  </si>
-  <si>
     <t>Absolute Neutrophil Count  ($10^9 cells/L$)</t>
   </si>
   <si>
@@ -728,15 +725,9 @@
     <t>ca199_0</t>
   </si>
   <si>
-    <t>**Longitudinal - Hematology**</t>
-  </si>
-  <si>
     <t>**Longitudinal - Chemistry**</t>
   </si>
   <si>
-    <t>**Longitudinal - Liver Function**</t>
-  </si>
-  <si>
     <t>**Longitudinal - Management**</t>
   </si>
   <si>
@@ -747,6 +738,15 @@
   </si>
   <si>
     <t>height_0</t>
+  </si>
+  <si>
+    <t>Serum Albumin (g/L)</t>
+  </si>
+  <si>
+    <t>**Longitudinal - CBC**</t>
+  </si>
+  <si>
+    <t>**Longitudinal - LFT**</t>
   </si>
 </sst>
 </file>
@@ -1534,7 +1534,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B19" t="s">
         <v>186</v>
@@ -1864,7 +1864,7 @@
     </row>
     <row r="34" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="G34">
         <v>33</v>
@@ -1872,7 +1872,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B35" t="s">
         <v>158</v>
@@ -1881,7 +1881,7 @@
         <v>77</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E35" t="s">
         <v>100</v>
@@ -1895,7 +1895,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B36" t="s">
         <v>149</v>
@@ -1904,7 +1904,7 @@
         <v>77</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E36" t="s">
         <v>101</v>
@@ -1918,7 +1918,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B37" t="s">
         <v>70</v>
@@ -1927,7 +1927,7 @@
         <v>77</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E37" t="s">
         <v>102</v>
@@ -1941,7 +1941,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B38" t="s">
         <v>187</v>
@@ -1950,7 +1950,7 @@
         <v>77</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E38" t="s">
         <v>104</v>
@@ -1964,7 +1964,7 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B39" t="s">
         <v>196</v>
@@ -1973,7 +1973,7 @@
         <v>77</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E39" t="s">
         <v>105</v>
@@ -1987,7 +1987,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B40" t="s">
         <v>197</v>
@@ -1996,7 +1996,7 @@
         <v>77</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E40" t="s">
         <v>106</v>
@@ -2010,7 +2010,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B41" t="s">
         <v>146</v>
@@ -2019,7 +2019,7 @@
         <v>77</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E41" t="s">
         <v>107</v>
@@ -2033,7 +2033,7 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B42" t="s">
         <v>142</v>
@@ -2042,7 +2042,7 @@
         <v>77</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E42" t="s">
         <v>109</v>
@@ -2056,7 +2056,7 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B43" t="s">
         <v>194</v>
@@ -2065,7 +2065,7 @@
         <v>77</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E43" t="s">
         <v>110</v>
@@ -2079,7 +2079,7 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B44" t="s">
         <v>195</v>
@@ -2088,7 +2088,7 @@
         <v>77</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E44" t="s">
         <v>111</v>
@@ -2102,7 +2102,7 @@
     </row>
     <row r="45" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="G45">
         <v>44</v>
@@ -2119,7 +2119,7 @@
         <v>77</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E46" t="s">
         <v>129</v>
@@ -2142,7 +2142,7 @@
         <v>77</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E47" t="s">
         <v>130</v>
@@ -2165,7 +2165,7 @@
         <v>77</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E48" t="s">
         <v>131</v>
@@ -2188,7 +2188,7 @@
         <v>77</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E49" t="s">
         <v>128</v>
@@ -2211,7 +2211,7 @@
         <v>77</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E50" t="s">
         <v>103</v>
@@ -2228,13 +2228,13 @@
         <v>33</v>
       </c>
       <c r="B51" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C51" t="s">
         <v>77</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E51" t="s">
         <v>127</v>
@@ -2257,7 +2257,7 @@
         <v>77</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E52" t="s">
         <v>119</v>
@@ -2271,7 +2271,7 @@
     </row>
     <row r="53" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="G53" s="1">
         <v>52</v>
@@ -2288,7 +2288,7 @@
         <v>77</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E54" t="s">
         <v>132</v>
@@ -2311,7 +2311,7 @@
         <v>77</v>
       </c>
       <c r="D55" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E55" t="s">
         <v>133</v>
@@ -2325,7 +2325,7 @@
     </row>
     <row r="56" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="G56" s="1">
         <v>55</v>
@@ -2342,7 +2342,7 @@
         <v>77</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E57" t="s">
         <v>134</v>
@@ -2359,13 +2359,13 @@
         <v>36</v>
       </c>
       <c r="B58" t="s">
-        <v>198</v>
+        <v>233</v>
       </c>
       <c r="C58" t="s">
         <v>77</v>
       </c>
       <c r="D58" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E58" t="s">
         <v>135</v>
@@ -2388,7 +2388,7 @@
         <v>77</v>
       </c>
       <c r="D59" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E59" t="s">
         <v>136</v>
@@ -2411,7 +2411,7 @@
         <v>77</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E60" t="s">
         <v>120</v>
@@ -2434,7 +2434,7 @@
         <v>77</v>
       </c>
       <c r="D61" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E61" t="s">
         <v>137</v>
@@ -2457,7 +2457,7 @@
         <v>77</v>
       </c>
       <c r="D62" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E62" t="s">
         <v>139</v>
@@ -2480,7 +2480,7 @@
         <v>77</v>
       </c>
       <c r="D63" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E63" t="s">
         <v>138</v>
@@ -2503,7 +2503,7 @@
         <v>77</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E64" t="s">
         <v>108</v>
@@ -2517,7 +2517,7 @@
     </row>
     <row r="65" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="G65" s="1">
         <v>64</v>
@@ -2580,7 +2580,7 @@
         <v>77</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E68" t="s">
         <v>123</v>
@@ -2626,7 +2626,7 @@
         <v>77</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E70" t="s">
         <v>125</v>
@@ -2663,27 +2663,27 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D73" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D74" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D75" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D76" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D77" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -2696,6 +2696,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000C8DD2C9503A9346957BF8010701C0C0" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8fb9d6bcbce96ea4820cba4545c13952">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="44ad9495-3741-4708-b440-876241155999" xmlns:ns3="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c86def3c84f9d4c2cb9156fbe4c263eb" ns2:_="" ns3:_="">
     <xsd:import namespace="44ad9495-3741-4708-b440-876241155999"/>
@@ -2930,15 +2939,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2951,6 +2951,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{351A9940-6E89-4EED-A102-125C210064C4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C54C97D-D015-4BC8-B84D-2E3C5CF96B75}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2969,14 +2977,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{351A9940-6E89-4EED-A102-125C210064C4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05141117-6D65-4604-9391-C80E4C64FB19}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat: Incorporate pt age into analysis
Imported age into `01_data-cleaning.qmd` from the supplemental CSV document provided by Dr. Mazhindu, and updated relevant chunks to include it in the analysis. Updated the data glossary spreadsheet to include age and associated meta information.

Added data validation for the step where several chemo type categories were combined.

Refs: MET-004, DAT-025
</commit_message>
<xml_diff>
--- a/docs/glossary.xlsx
+++ b/docs/glossary.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olucdenver.sharepoint.com/sites/HendricksLabDailyWorkSpace/Shared Documents/Research Projects/Tinashe Collaborations/gi-cancer_project/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dukec\Documents\gi-cancer_project_local\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="8_{074114E1-AEC4-440E-9A9F-2F76837AA4D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5837F166-8F3C-4710-B010-6AD1C8B582A4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E86238-7449-402E-91B9-B8CC165C2283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="61152" yWindow="3192" windowWidth="34560" windowHeight="18600" xr2:uid="{2AF94D29-0516-4E66-985C-E773281D9243}"/>
+    <workbookView xWindow="46104" yWindow="3744" windowWidth="34560" windowHeight="18648" xr2:uid="{2AF94D29-0516-4E66-985C-E773281D9243}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$72</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="240">
   <si>
     <t>Variable</t>
   </si>
@@ -747,6 +747,18 @@
   </si>
   <si>
     <t>**Longitudinal - LFT**</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>Age (years)</t>
+  </si>
+  <si>
+    <t>**Valid:** 18 - 100</t>
+  </si>
+  <si>
+    <t>`Age (years)`</t>
   </si>
 </sst>
 </file>
@@ -812,13 +824,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1153,7 +1166,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60F3F596-38F5-43D0-B51C-7C799C94B00A}">
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.5546875" bestFit="1" customWidth="1"/>
@@ -1161,6 +1174,8 @@
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="123.109375" customWidth="1"/>
     <col min="5" max="5" width="126.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.21875" customWidth="1"/>
+    <col min="7" max="7" width="20.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -1248,273 +1263,267 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D6" t="s">
-        <v>166</v>
-      </c>
-      <c r="E6" t="s">
-        <v>81</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="G6">
-        <v>5</v>
+    <row r="6" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C7" t="s">
         <v>163</v>
       </c>
       <c r="D7" t="s">
+        <v>166</v>
+      </c>
+      <c r="E7" t="s">
+        <v>81</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" t="s">
+        <v>163</v>
+      </c>
+      <c r="D8" t="s">
         <v>167</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E8" t="s">
         <v>82</v>
       </c>
-      <c r="F7">
+      <c r="F8">
         <v>5</v>
       </c>
-      <c r="G7">
+      <c r="G8">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+    <row r="9" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G9" s="1">
         <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>150</v>
-      </c>
-      <c r="C9" t="s">
-        <v>163</v>
-      </c>
-      <c r="D9" t="s">
-        <v>168</v>
-      </c>
-      <c r="E9" t="s">
-        <v>83</v>
-      </c>
-      <c r="F9">
-        <v>3</v>
-      </c>
-      <c r="G9">
-        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>150</v>
       </c>
       <c r="C10" t="s">
         <v>163</v>
       </c>
       <c r="D10" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F10">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G10">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C11" t="s">
         <v>163</v>
       </c>
       <c r="D11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F11">
-        <v>7</v>
-      </c>
-      <c r="G11" s="1">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="G11">
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>140</v>
+        <v>57</v>
       </c>
       <c r="C12" t="s">
         <v>163</v>
       </c>
       <c r="D12" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F12">
-        <v>8</v>
-      </c>
-      <c r="G12">
-        <v>11</v>
+        <v>7</v>
+      </c>
+      <c r="G12" s="1">
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="C13" t="s">
         <v>163</v>
       </c>
       <c r="D13" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E13" t="s">
-        <v>112</v>
+        <v>86</v>
       </c>
       <c r="F13">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="G13">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C14" t="s">
         <v>163</v>
       </c>
       <c r="D14" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="E14" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F14">
-        <v>47</v>
-      </c>
-      <c r="G14" s="1">
-        <v>13</v>
+        <v>46</v>
+      </c>
+      <c r="G14">
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C15" t="s">
         <v>163</v>
       </c>
       <c r="D15" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F15">
-        <v>48</v>
-      </c>
-      <c r="G15">
-        <v>14</v>
+        <v>47</v>
+      </c>
+      <c r="G15" s="1">
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C16" t="s">
         <v>163</v>
       </c>
       <c r="D16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F16">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G16">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C17" t="s">
-        <v>77</v>
+        <v>163</v>
       </c>
       <c r="D17" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E17" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F17">
-        <v>50</v>
-      </c>
-      <c r="G17" s="1">
-        <v>16</v>
+        <v>49</v>
+      </c>
+      <c r="G17">
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C18" t="s">
         <v>77</v>
@@ -1523,75 +1532,75 @@
         <v>177</v>
       </c>
       <c r="E18" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F18">
-        <v>51</v>
-      </c>
-      <c r="G18">
-        <v>17</v>
+        <v>50</v>
+      </c>
+      <c r="G18" s="1">
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" t="s">
+        <v>185</v>
+      </c>
+      <c r="C19" t="s">
+        <v>77</v>
+      </c>
+      <c r="D19" t="s">
+        <v>177</v>
+      </c>
+      <c r="E19" t="s">
+        <v>117</v>
+      </c>
+      <c r="F19">
+        <v>51</v>
+      </c>
+      <c r="G19">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>219</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B20" t="s">
         <v>186</v>
       </c>
-      <c r="C19" t="s">
-        <v>77</v>
-      </c>
-      <c r="D19" t="s">
+      <c r="C20" t="s">
+        <v>77</v>
+      </c>
+      <c r="D20" t="s">
         <v>178</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E20" t="s">
         <v>118</v>
       </c>
-      <c r="F19">
+      <c r="F20">
         <v>52</v>
       </c>
-      <c r="G19">
+      <c r="G20">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
+    <row r="21" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="G20" s="1">
+      <c r="G21" s="1">
         <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>9</v>
-      </c>
-      <c r="B21" t="s">
-        <v>58</v>
-      </c>
-      <c r="C21" t="s">
-        <v>163</v>
-      </c>
-      <c r="D21" t="s">
-        <v>175</v>
-      </c>
-      <c r="E21" t="s">
-        <v>87</v>
-      </c>
-      <c r="F21">
-        <v>9</v>
-      </c>
-      <c r="G21">
-        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B22" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C22" t="s">
         <v>163</v>
@@ -1600,21 +1609,21 @@
         <v>175</v>
       </c>
       <c r="E22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F22">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G22">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C23" t="s">
         <v>163</v>
@@ -1623,21 +1632,21 @@
         <v>175</v>
       </c>
       <c r="E23" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F23">
-        <v>11</v>
-      </c>
-      <c r="G23" s="1">
-        <v>22</v>
+        <v>10</v>
+      </c>
+      <c r="G23">
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C24" t="s">
         <v>163</v>
@@ -1646,21 +1655,21 @@
         <v>175</v>
       </c>
       <c r="E24" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F24">
-        <v>12</v>
-      </c>
-      <c r="G24">
-        <v>23</v>
+        <v>11</v>
+      </c>
+      <c r="G24" s="1">
+        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C25" t="s">
         <v>163</v>
@@ -1669,21 +1678,21 @@
         <v>175</v>
       </c>
       <c r="E25" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F25">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G25">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="C26" t="s">
         <v>163</v>
@@ -1692,21 +1701,21 @@
         <v>175</v>
       </c>
       <c r="E26" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F26">
-        <v>14</v>
-      </c>
-      <c r="G26" s="1">
-        <v>25</v>
+        <v>13</v>
+      </c>
+      <c r="G26">
+        <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B27" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="C27" t="s">
         <v>163</v>
@@ -1715,21 +1724,21 @@
         <v>175</v>
       </c>
       <c r="E27" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F27">
-        <v>15</v>
-      </c>
-      <c r="G27">
-        <v>26</v>
+        <v>14</v>
+      </c>
+      <c r="G27" s="1">
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C28" t="s">
         <v>163</v>
@@ -1738,21 +1747,21 @@
         <v>175</v>
       </c>
       <c r="E28" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F28">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G28">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B29" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C29" t="s">
         <v>163</v>
@@ -1761,21 +1770,21 @@
         <v>175</v>
       </c>
       <c r="E29" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F29">
-        <v>17</v>
-      </c>
-      <c r="G29" s="1">
-        <v>28</v>
+        <v>16</v>
+      </c>
+      <c r="G29">
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B30" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C30" t="s">
         <v>163</v>
@@ -1784,21 +1793,21 @@
         <v>175</v>
       </c>
       <c r="E30" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F30">
-        <v>18</v>
-      </c>
-      <c r="G30">
-        <v>29</v>
+        <v>17</v>
+      </c>
+      <c r="G30" s="1">
+        <v>28</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B31" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C31" t="s">
         <v>163</v>
@@ -1807,21 +1816,21 @@
         <v>175</v>
       </c>
       <c r="E31" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F31">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G31">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B32" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C32" t="s">
         <v>163</v>
@@ -1830,75 +1839,75 @@
         <v>175</v>
       </c>
       <c r="E32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F32">
-        <v>20</v>
-      </c>
-      <c r="G32" s="1">
-        <v>31</v>
+        <v>19</v>
+      </c>
+      <c r="G32">
+        <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" t="s">
+        <v>68</v>
+      </c>
+      <c r="C33" t="s">
+        <v>163</v>
+      </c>
+      <c r="D33" t="s">
+        <v>175</v>
+      </c>
+      <c r="E33" t="s">
+        <v>98</v>
+      </c>
+      <c r="F33">
+        <v>20</v>
+      </c>
+      <c r="G33" s="1">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
         <v>27</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>76</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C34" t="s">
         <v>164</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D34" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E34" t="s">
         <v>99</v>
       </c>
-      <c r="F33">
+      <c r="F34">
         <v>78</v>
       </c>
-      <c r="G33">
+      <c r="G34">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
+    <row r="35" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="G34">
+      <c r="G35">
         <v>33</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>231</v>
-      </c>
-      <c r="B35" t="s">
-        <v>158</v>
-      </c>
-      <c r="C35" t="s">
-        <v>77</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="E35" t="s">
-        <v>100</v>
-      </c>
-      <c r="F35">
-        <v>21</v>
-      </c>
-      <c r="G35" s="1">
-        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B36" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="C36" t="s">
         <v>77</v>
@@ -1907,67 +1916,67 @@
         <v>207</v>
       </c>
       <c r="E36" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F36">
-        <v>22</v>
-      </c>
-      <c r="G36">
-        <v>35</v>
+        <v>21</v>
+      </c>
+      <c r="G36" s="1">
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="B37" t="s">
-        <v>70</v>
+        <v>149</v>
       </c>
       <c r="C37" t="s">
         <v>77</v>
       </c>
-      <c r="D37" s="5" t="s">
-        <v>218</v>
+      <c r="D37" s="2" t="s">
+        <v>207</v>
       </c>
       <c r="E37" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F37">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G37">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B38" t="s">
-        <v>187</v>
+        <v>70</v>
       </c>
       <c r="C38" t="s">
         <v>77</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>200</v>
+      <c r="D38" s="5" t="s">
+        <v>218</v>
       </c>
       <c r="E38" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F38">
-        <v>27</v>
-      </c>
-      <c r="G38" s="1">
-        <v>37</v>
+        <v>23</v>
+      </c>
+      <c r="G38">
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B39" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="C39" t="s">
         <v>77</v>
@@ -1976,21 +1985,21 @@
         <v>200</v>
       </c>
       <c r="E39" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F39">
-        <v>33</v>
-      </c>
-      <c r="G39">
-        <v>38</v>
+        <v>27</v>
+      </c>
+      <c r="G39" s="1">
+        <v>37</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B40" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C40" t="s">
         <v>77</v>
@@ -1999,21 +2008,21 @@
         <v>200</v>
       </c>
       <c r="E40" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F40">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G40">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B41" t="s">
-        <v>146</v>
+        <v>197</v>
       </c>
       <c r="C41" t="s">
         <v>77</v>
@@ -2022,21 +2031,21 @@
         <v>200</v>
       </c>
       <c r="E41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F41">
-        <v>35</v>
-      </c>
-      <c r="G41" s="1">
-        <v>40</v>
+        <v>34</v>
+      </c>
+      <c r="G41">
+        <v>39</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B42" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C42" t="s">
         <v>77</v>
@@ -2045,21 +2054,21 @@
         <v>200</v>
       </c>
       <c r="E42" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F42">
-        <v>43</v>
-      </c>
-      <c r="G42">
-        <v>41</v>
+        <v>35</v>
+      </c>
+      <c r="G42" s="1">
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B43" t="s">
-        <v>194</v>
+        <v>142</v>
       </c>
       <c r="C43" t="s">
         <v>77</v>
@@ -2068,21 +2077,21 @@
         <v>200</v>
       </c>
       <c r="E43" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F43">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G43">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B44" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C44" t="s">
         <v>77</v>
@@ -2091,75 +2100,75 @@
         <v>200</v>
       </c>
       <c r="E44" t="s">
+        <v>110</v>
+      </c>
+      <c r="F44">
+        <v>44</v>
+      </c>
+      <c r="G44">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>227</v>
+      </c>
+      <c r="B45" t="s">
+        <v>195</v>
+      </c>
+      <c r="C45" t="s">
+        <v>77</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="E45" t="s">
         <v>111</v>
       </c>
-      <c r="F44">
+      <c r="F45">
         <v>45</v>
       </c>
-      <c r="G44" s="1">
+      <c r="G45" s="1">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="1" t="s">
+    <row r="46" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="G45">
+      <c r="G46">
         <v>44</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>28</v>
-      </c>
-      <c r="B46" t="s">
-        <v>160</v>
-      </c>
-      <c r="C46" t="s">
-        <v>77</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="E46" t="s">
-        <v>129</v>
-      </c>
-      <c r="F46">
-        <v>28</v>
-      </c>
-      <c r="G46">
-        <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B47" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="C47" t="s">
         <v>77</v>
       </c>
-      <c r="D47" s="2" t="s">
-        <v>200</v>
+      <c r="D47" s="3" t="s">
+        <v>199</v>
       </c>
       <c r="E47" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F47">
-        <v>29</v>
-      </c>
-      <c r="G47" s="1">
-        <v>46</v>
+        <v>28</v>
+      </c>
+      <c r="G47">
+        <v>45</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B48" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C48" t="s">
         <v>77</v>
@@ -2168,390 +2177,390 @@
         <v>200</v>
       </c>
       <c r="E48" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F48">
-        <v>30</v>
-      </c>
-      <c r="G48">
-        <v>47</v>
+        <v>29</v>
+      </c>
+      <c r="G48" s="1">
+        <v>46</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B49" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C49" t="s">
         <v>77</v>
       </c>
-      <c r="D49" s="3" t="s">
-        <v>208</v>
+      <c r="D49" s="2" t="s">
+        <v>200</v>
       </c>
       <c r="E49" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="F49">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G49">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B50" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="C50" t="s">
         <v>77</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="E50" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="F50">
-        <v>24</v>
-      </c>
-      <c r="G50" s="1">
-        <v>49</v>
+        <v>26</v>
+      </c>
+      <c r="G50">
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B51" t="s">
-        <v>198</v>
+        <v>141</v>
       </c>
       <c r="C51" t="s">
         <v>77</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="E51" t="s">
-        <v>127</v>
+        <v>103</v>
       </c>
       <c r="F51">
-        <v>25</v>
-      </c>
-      <c r="G51">
-        <v>50</v>
+        <v>24</v>
+      </c>
+      <c r="G51" s="1">
+        <v>49</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
+        <v>33</v>
+      </c>
+      <c r="B52" t="s">
+        <v>198</v>
+      </c>
+      <c r="C52" t="s">
+        <v>77</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="E52" t="s">
+        <v>127</v>
+      </c>
+      <c r="F52">
+        <v>25</v>
+      </c>
+      <c r="G52">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
         <v>34</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B53" t="s">
         <v>151</v>
       </c>
-      <c r="C52" t="s">
-        <v>77</v>
-      </c>
-      <c r="D52" s="3" t="s">
+      <c r="C53" t="s">
+        <v>77</v>
+      </c>
+      <c r="D53" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="E52" t="s">
+      <c r="E53" t="s">
         <v>119</v>
       </c>
-      <c r="F52">
+      <c r="F53">
         <v>60</v>
       </c>
-      <c r="G52">
+      <c r="G53">
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="1" t="s">
+    <row r="54" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="G53" s="1">
+      <c r="G54" s="1">
         <v>52</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>43</v>
-      </c>
-      <c r="B54" t="s">
-        <v>159</v>
-      </c>
-      <c r="C54" t="s">
-        <v>77</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="E54" t="s">
-        <v>132</v>
-      </c>
-      <c r="F54">
-        <v>31</v>
-      </c>
-      <c r="G54">
-        <v>53</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
+        <v>43</v>
+      </c>
+      <c r="B55" t="s">
+        <v>159</v>
+      </c>
+      <c r="C55" t="s">
+        <v>77</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="E55" t="s">
+        <v>132</v>
+      </c>
+      <c r="F55">
+        <v>31</v>
+      </c>
+      <c r="G55">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
         <v>44</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B56" t="s">
         <v>155</v>
       </c>
-      <c r="C55" t="s">
-        <v>77</v>
-      </c>
-      <c r="D55" t="s">
+      <c r="C56" t="s">
+        <v>77</v>
+      </c>
+      <c r="D56" t="s">
         <v>209</v>
       </c>
-      <c r="E55" t="s">
+      <c r="E56" t="s">
         <v>133</v>
       </c>
-      <c r="F55">
+      <c r="F56">
         <v>32</v>
       </c>
-      <c r="G55">
+      <c r="G56">
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="1" t="s">
+    <row r="57" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="G56" s="1">
+      <c r="G57" s="1">
         <v>55</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>35</v>
-      </c>
-      <c r="B57" t="s">
-        <v>157</v>
-      </c>
-      <c r="C57" t="s">
-        <v>77</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="E57" t="s">
-        <v>134</v>
-      </c>
-      <c r="F57">
-        <v>36</v>
-      </c>
-      <c r="G57">
-        <v>56</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
+        <v>35</v>
+      </c>
+      <c r="B58" t="s">
+        <v>157</v>
+      </c>
+      <c r="C58" t="s">
+        <v>77</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="E58" t="s">
+        <v>134</v>
+      </c>
+      <c r="F58">
         <v>36</v>
       </c>
-      <c r="B58" t="s">
-        <v>233</v>
-      </c>
-      <c r="C58" t="s">
-        <v>77</v>
-      </c>
-      <c r="D58" t="s">
-        <v>201</v>
-      </c>
-      <c r="E58" t="s">
-        <v>135</v>
-      </c>
-      <c r="F58">
-        <v>37</v>
-      </c>
       <c r="G58">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
+        <v>36</v>
+      </c>
+      <c r="B59" t="s">
+        <v>233</v>
+      </c>
+      <c r="C59" t="s">
+        <v>77</v>
+      </c>
+      <c r="D59" t="s">
+        <v>201</v>
+      </c>
+      <c r="E59" t="s">
+        <v>135</v>
+      </c>
+      <c r="F59">
         <v>37</v>
       </c>
-      <c r="B59" t="s">
-        <v>156</v>
-      </c>
-      <c r="C59" t="s">
-        <v>77</v>
-      </c>
-      <c r="D59" t="s">
-        <v>211</v>
-      </c>
-      <c r="E59" t="s">
-        <v>136</v>
-      </c>
-      <c r="F59">
-        <v>38</v>
-      </c>
-      <c r="G59" s="1">
-        <v>58</v>
+      <c r="G59">
+        <v>57</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
+        <v>37</v>
+      </c>
+      <c r="B60" t="s">
+        <v>156</v>
+      </c>
+      <c r="C60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D60" t="s">
+        <v>211</v>
+      </c>
+      <c r="E60" t="s">
+        <v>136</v>
+      </c>
+      <c r="F60">
         <v>38</v>
       </c>
-      <c r="B60" t="s">
-        <v>147</v>
-      </c>
-      <c r="C60" t="s">
-        <v>77</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="E60" t="s">
-        <v>120</v>
-      </c>
-      <c r="F60">
-        <v>67</v>
-      </c>
-      <c r="G60">
-        <v>59</v>
+      <c r="G60" s="1">
+        <v>58</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B61" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C61" t="s">
         <v>77</v>
       </c>
-      <c r="D61" t="s">
-        <v>202</v>
+      <c r="D61" s="2" t="s">
+        <v>200</v>
       </c>
       <c r="E61" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
       <c r="F61">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="G61">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B62" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C62" t="s">
         <v>77</v>
       </c>
       <c r="D62" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E62" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F62">
-        <v>41</v>
-      </c>
-      <c r="G62" s="1">
-        <v>61</v>
+        <v>39</v>
+      </c>
+      <c r="G62">
+        <v>60</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
+        <v>40</v>
+      </c>
+      <c r="B63" t="s">
+        <v>144</v>
+      </c>
+      <c r="C63" t="s">
+        <v>77</v>
+      </c>
+      <c r="D63" t="s">
+        <v>203</v>
+      </c>
+      <c r="E63" t="s">
+        <v>139</v>
+      </c>
+      <c r="F63">
         <v>41</v>
       </c>
-      <c r="B63" t="s">
-        <v>145</v>
-      </c>
-      <c r="C63" t="s">
-        <v>77</v>
-      </c>
-      <c r="D63" t="s">
-        <v>205</v>
-      </c>
-      <c r="E63" t="s">
-        <v>138</v>
-      </c>
-      <c r="F63">
-        <v>40</v>
-      </c>
-      <c r="G63">
-        <v>62</v>
+      <c r="G63" s="1">
+        <v>61</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
+        <v>41</v>
+      </c>
+      <c r="B64" t="s">
+        <v>145</v>
+      </c>
+      <c r="C64" t="s">
+        <v>77</v>
+      </c>
+      <c r="D64" t="s">
+        <v>205</v>
+      </c>
+      <c r="E64" t="s">
+        <v>138</v>
+      </c>
+      <c r="F64">
+        <v>40</v>
+      </c>
+      <c r="G64">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
         <v>42</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B65" t="s">
         <v>148</v>
       </c>
-      <c r="C64" t="s">
-        <v>77</v>
-      </c>
-      <c r="D64" s="2" t="s">
+      <c r="C65" t="s">
+        <v>77</v>
+      </c>
+      <c r="D65" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="E64" t="s">
+      <c r="E65" t="s">
         <v>108</v>
       </c>
-      <c r="F64">
+      <c r="F65">
         <v>42</v>
       </c>
-      <c r="G64">
+      <c r="G65">
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="1" t="s">
+    <row r="66" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="G65" s="1">
+      <c r="G66" s="1">
         <v>64</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
-        <v>45</v>
-      </c>
-      <c r="B66" t="s">
-        <v>188</v>
-      </c>
-      <c r="C66" t="s">
-        <v>163</v>
-      </c>
-      <c r="D66" t="s">
-        <v>175</v>
-      </c>
-      <c r="E66" t="s">
-        <v>121</v>
-      </c>
-      <c r="F66">
-        <v>72</v>
-      </c>
-      <c r="G66">
-        <v>65</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B67" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C67" t="s">
         <v>163</v>
@@ -2560,148 +2569,173 @@
         <v>175</v>
       </c>
       <c r="E67" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F67">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G67">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B68" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C68" t="s">
-        <v>77</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>207</v>
+        <v>163</v>
+      </c>
+      <c r="D68" t="s">
+        <v>175</v>
       </c>
       <c r="E68" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F68">
-        <v>74</v>
-      </c>
-      <c r="G68" s="1">
-        <v>67</v>
+        <v>73</v>
+      </c>
+      <c r="G68">
+        <v>66</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B69" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C69" t="s">
-        <v>163</v>
-      </c>
-      <c r="D69" t="s">
-        <v>175</v>
+        <v>77</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>207</v>
       </c>
       <c r="E69" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F69">
-        <v>75</v>
-      </c>
-      <c r="G69">
-        <v>68</v>
+        <v>74</v>
+      </c>
+      <c r="G69" s="1">
+        <v>67</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B70" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C70" t="s">
-        <v>77</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>207</v>
+        <v>163</v>
+      </c>
+      <c r="D70" t="s">
+        <v>175</v>
       </c>
       <c r="E70" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F70">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G70">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
+        <v>49</v>
+      </c>
+      <c r="B71" t="s">
+        <v>192</v>
+      </c>
+      <c r="C71" t="s">
+        <v>77</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="E71" t="s">
+        <v>125</v>
+      </c>
+      <c r="F71">
+        <v>76</v>
+      </c>
+      <c r="G71">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
         <v>50</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B72" t="s">
         <v>193</v>
       </c>
-      <c r="C71" t="s">
+      <c r="C72" t="s">
         <v>163</v>
       </c>
-      <c r="D71" t="s">
+      <c r="D72" t="s">
         <v>175</v>
       </c>
-      <c r="E71" t="s">
+      <c r="E72" t="s">
         <v>126</v>
       </c>
-      <c r="F71">
-        <v>77</v>
-      </c>
-      <c r="G71" s="1">
+      <c r="F72">
+        <v>77</v>
+      </c>
+      <c r="G72" s="1">
         <v>70</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D73" s="3" t="s">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D74" s="3" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D74" s="2" t="s">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D75" s="2" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D75" s="4" t="s">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D76" s="4" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D76" s="5" t="s">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D77" s="5" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D77" t="s">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D78" t="s">
         <v>217</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G71" xr:uid="{60F3F596-38F5-43D0-B51C-7C799C94B00A}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A64:G64">
-    <sortCondition ref="A64"/>
+  <autoFilter ref="A1:G72" xr:uid="{60F3F596-38F5-43D0-B51C-7C799C94B00A}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A65:G65">
+    <sortCondition ref="A65"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="44ad9495-3741-4708-b440-876241155999">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2940,20 +2974,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="44ad9495-3741-4708-b440-876241155999">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{351A9940-6E89-4EED-A102-125C210064C4}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05141117-6D65-4604-9391-C80E4C64FB19}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="44ad9495-3741-4708-b440-876241155999"/>
+    <ds:schemaRef ds:uri="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2978,12 +3013,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05141117-6D65-4604-9391-C80E4C64FB19}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{351A9940-6E89-4EED-A102-125C210064C4}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="44ad9495-3741-4708-b440-876241155999"/>
-    <ds:schemaRef ds:uri="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore: add sex to glossary documents
</commit_message>
<xml_diff>
--- a/docs/glossary.xlsx
+++ b/docs/glossary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dukec\Documents\gi-cancer_project_local\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\E. Duke Chase\Documents\gi-cancer_project_local\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E86238-7449-402E-91B9-B8CC165C2283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F460E1CF-F51B-4FE3-8064-E53954A48B9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46104" yWindow="3744" windowWidth="34560" windowHeight="18648" xr2:uid="{2AF94D29-0516-4E66-985C-E773281D9243}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{2AF94D29-0516-4E66-985C-E773281D9243}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -755,10 +755,10 @@
     <t>Age (years)</t>
   </si>
   <si>
-    <t>**Valid:** 18 - 100</t>
-  </si>
-  <si>
     <t>`Age (years)`</t>
+  </si>
+  <si>
+    <t>**Valid:** 18 - 120</t>
   </si>
 </sst>
 </file>
@@ -824,14 +824,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1167,18 +1166,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60F3F596-38F5-43D0-B51C-7C799C94B00A}">
   <dimension ref="A1:G78"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="43" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="123.109375" customWidth="1"/>
-    <col min="5" max="5" width="126.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.21875" customWidth="1"/>
-    <col min="7" max="7" width="20.88671875" customWidth="1"/>
+    <col min="4" max="4" width="123.08984375" customWidth="1"/>
+    <col min="5" max="5" width="126.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.1796875" customWidth="1"/>
+    <col min="7" max="7" width="20.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1201,7 +1200,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>73</v>
       </c>
@@ -1209,7 +1208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1232,7 +1231,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1255,7 +1254,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>74</v>
       </c>
@@ -1263,24 +1262,24 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>236</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" t="s">
         <v>237</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="D6" s="6" t="s">
+      <c r="C6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" t="s">
+        <v>239</v>
+      </c>
+      <c r="E6" t="s">
         <v>238</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1303,7 +1302,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -1326,7 +1325,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>75</v>
       </c>
@@ -1334,7 +1333,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1357,7 +1356,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1380,7 +1379,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -1403,7 +1402,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -1426,7 +1425,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -1449,7 +1448,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -1472,7 +1471,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -1495,7 +1494,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -1518,7 +1517,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -1541,7 +1540,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -1564,7 +1563,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>219</v>
       </c>
@@ -1587,7 +1586,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>162</v>
       </c>
@@ -1595,7 +1594,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -1618,7 +1617,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -1641,7 +1640,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -1664,7 +1663,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -1687,7 +1686,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>13</v>
       </c>
@@ -1710,7 +1709,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>14</v>
       </c>
@@ -1733,7 +1732,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>15</v>
       </c>
@@ -1756,7 +1755,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>16</v>
       </c>
@@ -1779,7 +1778,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>17</v>
       </c>
@@ -1802,7 +1801,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>18</v>
       </c>
@@ -1825,7 +1824,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>19</v>
       </c>
@@ -1848,7 +1847,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>20</v>
       </c>
@@ -1871,7 +1870,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>27</v>
       </c>
@@ -1894,7 +1893,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>230</v>
       </c>
@@ -1902,7 +1901,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>231</v>
       </c>
@@ -1925,7 +1924,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>232</v>
       </c>
@@ -1948,7 +1947,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>220</v>
       </c>
@@ -1971,7 +1970,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>221</v>
       </c>
@@ -1994,7 +1993,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>222</v>
       </c>
@@ -2017,7 +2016,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>223</v>
       </c>
@@ -2040,7 +2039,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>224</v>
       </c>
@@ -2063,7 +2062,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>225</v>
       </c>
@@ -2086,7 +2085,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>226</v>
       </c>
@@ -2109,7 +2108,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>227</v>
       </c>
@@ -2132,7 +2131,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>234</v>
       </c>
@@ -2140,7 +2139,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>28</v>
       </c>
@@ -2163,7 +2162,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>29</v>
       </c>
@@ -2186,7 +2185,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>30</v>
       </c>
@@ -2209,7 +2208,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>31</v>
       </c>
@@ -2232,7 +2231,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>32</v>
       </c>
@@ -2255,7 +2254,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>33</v>
       </c>
@@ -2278,7 +2277,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>34</v>
       </c>
@@ -2301,7 +2300,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="54" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>228</v>
       </c>
@@ -2309,7 +2308,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>43</v>
       </c>
@@ -2332,7 +2331,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>44</v>
       </c>
@@ -2355,7 +2354,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="57" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>235</v>
       </c>
@@ -2363,7 +2362,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>35</v>
       </c>
@@ -2386,7 +2385,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>36</v>
       </c>
@@ -2409,7 +2408,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>37</v>
       </c>
@@ -2432,7 +2431,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>38</v>
       </c>
@@ -2455,7 +2454,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>39</v>
       </c>
@@ -2478,7 +2477,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>40</v>
       </c>
@@ -2501,7 +2500,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>41</v>
       </c>
@@ -2524,7 +2523,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>42</v>
       </c>
@@ -2547,7 +2546,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="66" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>229</v>
       </c>
@@ -2555,7 +2554,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>45</v>
       </c>
@@ -2578,7 +2577,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>46</v>
       </c>
@@ -2601,7 +2600,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>47</v>
       </c>
@@ -2624,7 +2623,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>48</v>
       </c>
@@ -2647,7 +2646,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>49</v>
       </c>
@@ -2670,7 +2669,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>50</v>
       </c>
@@ -2693,27 +2692,27 @@
         <v>70</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D74" s="3" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D75" s="2" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D76" s="4" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D77" s="5" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D78" t="s">
         <v>217</v>
       </c>
@@ -2728,19 +2727,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="44ad9495-3741-4708-b440-876241155999">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000C8DD2C9503A9346957BF8010701C0C0" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8fb9d6bcbce96ea4820cba4545c13952">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="44ad9495-3741-4708-b440-876241155999" xmlns:ns3="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c86def3c84f9d4c2cb9156fbe4c263eb" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000C8DD2C9503A9346957BF8010701C0C0" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="36c570434a73bd4724d1e0329b0da23d">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="44ad9495-3741-4708-b440-876241155999" xmlns:ns3="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="15d4c143b1ef6d1abf62619997e119eb" ns2:_="" ns3:_="">
     <xsd:import namespace="44ad9495-3741-4708-b440-876241155999"/>
     <xsd:import namespace="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7"/>
     <xsd:element name="properties">
@@ -2973,6 +2961,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="44ad9495-3741-4708-b440-876241155999">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2983,18 +2982,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05141117-6D65-4604-9391-C80E4C64FB19}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="44ad9495-3741-4708-b440-876241155999"/>
-    <ds:schemaRef ds:uri="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C54C97D-D015-4BC8-B84D-2E3C5CF96B75}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A8367F6-0C7D-47A3-BF6F-0B8D204D7631}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -3012,6 +3000,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05141117-6D65-4604-9391-C80E4C64FB19}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="44ad9495-3741-4708-b440-876241155999"/>
+    <ds:schemaRef ds:uri="98305de1-6b4d-4e48-ba1d-6a2d8f079fc7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{351A9940-6E89-4EED-A102-125C210064C4}">
   <ds:schemaRefs>

</xml_diff>